<commit_message>
Reorganize: independent sport systems (fb/tt/bb naming, separate .env + monitoring per sport)
</commit_message>
<xml_diff>
--- a/table_tennis/data/tt_quasi_ml.xlsx
+++ b/table_tennis/data/tt_quasi_ml.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2670,6 +2670,126 @@
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:04:03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Maksiuta, Volodymyr</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Hrytsenko, Evhenii</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Setka Cup</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="K38" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Sportybet, 1xBet</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:04:03</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Maksiuta, Volodymyr</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Hrytsenko, Evhenii</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Setka Cup</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="K39" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Football.com, 1xBet</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>